<commit_message>
Sync most-advanced local replication tree (v1.2+ working state)
</commit_message>
<xml_diff>
--- a/extenbooks/AS001.xlsx
+++ b/extenbooks/AS001.xlsx
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -874,7 +874,11 @@
           <t>Chapter</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -916,7 +920,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1948–2024</t>
+          <t>1948-1989</t>
         </is>
       </c>
     </row>
@@ -928,7 +932,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>validated_book_and_extension</t>
+          <t>book_period_validated</t>
         </is>
       </c>
     </row>
@@ -970,78 +974,87 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Subseries</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>source / role</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AS001-A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>DPR (markdown)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t># AS001 — Social Burden Rate (b = 1 - Pn/S*)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>**Status**: validated_book_and_extension</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t># AS001 — Social Burden Rate (b = T/S* + Eu/S* = 1 − Pn/S*)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>**Chapter**: 7 central. **Units**: ratio.</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>## Series</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>## Definition</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>- **SID**: AS001</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Decomposes surplus value into the fraction reinvested as productive capital (Pn/S*) vs the fraction absorbed by state taxes (T/S*) and unproductive expenses (Eu/S*).</t>
+          <t>- **Name**: Social Burden Rate</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>- **Chapter**: Anu-Original Analytical (registry chapter=0 / null in research JSON). **AS-prefix framing**: this is a framework-derived analytical series, not a direct book-table replication. The conceptual home is the book's Ch7 §7.1 derivation of `r'n = (1 − b) r*'`, with `b = t + eu = T/S* + Eu/S*`.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  S* = Pn + T + Eu</t>
+          <t>- **Status**: `book_period_validated`</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1062,7 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  b  = (T + Eu)/S* = 1 - Pn/S*</t>
+          <t>- **Units**: ratio</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1074,7 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Book finding 1948-1989: b rises 0.56 → 0.66 (16% increase) — workers' surplus increasingly absorbed by state and unproductive activities.</t>
+          <t>## Methodology</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1086,7 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>## Construction</t>
+          <t>AS001 operationalizes the social burden rate from Shaikh &amp; Tonak's Ch7 §7.1 decomposition of surplus value. The book defines the relation `r'n = [1 − T/S* − Eu/S*][S*/(K*.u)] = (1 − t − eu) r*' = (1 − b) r*'`, where `r*' = S*/(K*.u)` is the capacity-utilization-adjusted Marxian rate of profit, `r'n = Pn/(K*.u)` is the similarly adjusted NIPA-based net rate of profit, `t = T/S*` is the tax share of surplus value, `eu = Eu/S*` is the unproductive-expenses share of surplus value, and `b = t + eu` is the social burden rate. The verbatim foundation is **"Divide equation (1) by utilized capital K*.u: r'n = [1 − T/S* − Eu/S*][S*/(K*.u)] = (1−t−eu)r*' = (1−b)r*'. Where r*' = S*/(K*.u) = capacity utilization-adjusted Marxian rate of profit; r'n = Pn/(K*.u) = similarly adjusted NIPA-based net rate of profit; t = T/S* = tax share of surplus value; eu = Eu/S* = unproductive expenses share of surplus value; b = t + eu = social burden rate."** (ST 1994 Ch7 §7.1, p.213). The interpretive anchor is **"Observed net rate of profit r'n will fall relative to Marxian general rate r*' when greater proportion of surplus value absorbed in business taxes or unproductive expenses. Hence: b = social burden rate."** (ST 1994 Ch7 §7.1, p.213).</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1098,7 @@
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pn approximation: NIPA 1.7.5 Line 17 (Corporate profits with IVA and CCAdj). This is TOTAL corporate profits; a more faithful Pn would apply the productive/unproductive concordance.</t>
+          <t>The construction rearranges the identity: `S* = Pn + T + Eu`, so `b = 1 − Pn/S*` is the fraction of surplus value not reinvested as productive capital. The Wave-1 implementation uses `Pn` approximated by NIPA Table 1.7.5 Line 17 (Corporate profits with IVA and CCAdj). This is total corporate profits; a fully faithful Pn would apply the productive/unproductive concordance from Appendix F to remove financial-sector profits. `S*` is taken from S505 (the project's Marxian surplus value series). `b = 1 − Pn/S505` is then computed annually 1948-2024. The legacy script is `code/A##_analytical/A07_social_burden_rate.py`. The book's headline empirical finding for the book period is **"Figure 7.1 shows the corresponding rise of 16% in social burden rate b over postwar period. Figure 7.2 result: NIPA-based rate rn falls substantially faster than Marxian rate. Marxian rate falls 25%, NIPA-based rate falls 39%."** (ST 1994 Ch7 §7.1, p.214). The book's reported b values rise from 0.56 (1948) to 0.66 (1989) — a 16% increase. Our implementation reports 0.7906 (1948) → 0.8577 (1989), magnitudes higher than the book by ~25 percentage points but directionally identical (RISING).</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1110,7 @@
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>S* = S505. b = 1 - Pn/S505.</t>
+          <t>The magnitude gap traces to two known approximations. First, our Pn (NIPA Line 17) undercounts S&amp;T's productive Pn (book's IVA-adjusted productive profits) because it lacks the productive/unproductive concordance. Second, without the concordance some financial-sector profit ends up in our Pn but not in the book's. Both issues bias `b = 1 − Pn/S*` upward (higher Pn → lower b; lower Pn → higher b — but the way our Pn is "wrong" combines an inflated numerator with an inflated S505 denominator, so the net effect is a moderately uniform upward bias). The directional finding — `b` rising over the postwar period — is what AS001's validator enforces and what the book's central social-burden-rate claim turns on. AS001's role in the S901 summary table is to expose the mechanism: when `b` rises, the NIPA-based profit rate falls faster than the Marxian rate, exactly as Figures 7.1-7.2 of the book document. The cross-link to S607/S608 (Net Social Wage) is via Appendix N's net-transfer concept — **"Net transfer: NT = Benefits received by workers − Taxes paid by workers. … Finding: Net transfer is negative over most of 1952-85 period → net tax on workers."** (ST 1994 Appendix N, pp.352-353).</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1122,7 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>## Findings (with caveat)</t>
+          <t>## Sources</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1134,7 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1948: b = 0.7906; 1989: b = 0.8577. **Direction: RISING** (book finding confirmed). Magnitudes higher than book's 0.56-0.66 because:</t>
+          <t>- KB chunks: `Inputs/Shaikh Tonak/Knowledge_Base/HDARP_Extractions/1994_Measuring_Wealth/chunk_24/full_transcription.md` (Ch7 §7.1 p.213-214 — formal definition `b = t + eu`, Figure 7.1 numeric finding, Figure 7.2 NIPA-Marxian gap); `chunk_35/full_transcription.md` (Appendix I Table I.1 — rates of exploitation of productive/unproductive workers, related decomposition); `chunk_38/full_transcription.md` (Appendix N — net transfer methodology, negative throughout postwar)</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1142,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1. Our Pn approximation undercounts S&amp;T's productive Pn (NIPA Line 17 vs Book's IVA-adjusted productive profits)</t>
+          <t>- Book tables: Ch7 §7.1 equations p.213; Figure 7.1 (social burden rate trajectory); Figure 7.2 (Marxian vs NIPA rate of profit); Appendix N Table N.2 (net transfer)</t>
         </is>
       </c>
     </row>
@@ -1137,19 +1150,23 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2. Without concordance, some financial-sector profit ends up in our Pn but not the book's</t>
+          <t>- External sources: BEA NIPA Table 1.7.5 Line 17 (Corporate profits with IVA and CCAdj) — cached locally 1929-2024</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>- Upstream series: S505 (Marxian surplus value S*), S607 (Net Social Wage, conceptual cross-link)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Directional finding PASSES. Magnitude refinement awaits IMPLEMENTATION_PLAN.md Phase 2.A (concordance) — at which point we re-apportion Line 17 to get strictly productive Pn.</t>
+          <t>- Code: `code/A##_analytical/A07_social_burden_rate.py` (legacy standalone analytical script — predates the standard L01/P02/V03 triad; flagged for migration in Stage 5)</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1178,7 @@
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>## Validator PASS</t>
+          <t>## Reference values</t>
         </is>
       </c>
     </row>
@@ -1173,31 +1190,207 @@
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Rising trend 1948→1989 confirmed (the book's qualitative finding).</t>
+          <t>- **Book period (validator-enforced)**: `b` rising 0.56 → 0.66 over 1948-1989 (book's Figure 7.1 finding; ~16% increase)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>- **Our implementation**: `b = 0.7906` (1948), `b = 0.8577` (1989), +8.5pp rise — magnitude offset ~25pp, direction matches</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>- **Validator `expected_range`**: `[0.3, 0.95]` (registry; share_series tolerance class)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>- **Direction**: monotonic rise 1948→1989 (PASS)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
-          <t>*Generated by anu-ingestion.*</t>
+          <t>- **Mechanism check**: r'n / r*' = (1 − b); with rising b, this ratio falls — and the book reports r'n falling 39% vs r*' falling 25%, consistent with b rising ~16%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>- **Extension period 1990-2024**: AS001 covers the full window (registry year_range 1948-2024) because both NIPA Line 17 and S505 extend; direction continues to rise modestly</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>## Known issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>- **Pn approximation**: our Pn = NIPA Line 17 (Corporate profits with IVA and CCAdj) is TOTAL corporate profits; a faithful Pn would apply the productive/unproductive concordance from Appendix F to remove financial-sector profits</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>- **Magnitude offset**: implementation reports b ~0.79-0.86 vs book's 0.56-0.66 — direction matches (rising) but levels are ~25pp higher; resolution awaits IMPLEMENTATION_PLAN.md Phase 2.A (concordance work), at which point Line 17 can be re-apportioned to strictly productive Pn</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>- **S505 dependency**: any drift in the upstream Marxian surplus value series propagates here</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>- **Legacy script not yet migrated** to the standard L01_AS001 / P02_AS001 / V03_AS001 triad; the construction array in the registry is empty for this reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>- **Construction array empty in registry**: signals "handled by legacy analytical script" rather than the standard pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>- **No EPR yet authored** for AS001 (Stage 4 work)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>## Cross-references</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>- Upstream: S505 (Marxian surplus value), NIPA Table 1.7.5 Line 17 (Pn proxy), S607 (Net Social Wage; conceptual link via Appendix N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>- Related decompositions: S506 (rate of surplus value e = S*/V*); S513 (Marxian profit rate r*); S514 (capacity-adjusted r*); AS002 (Khanjian cross-validation — same family of analytical consistency checks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>- Downstream: S901 (Chapter-9-style summary table; uses AS001 as the b component implicitly via the r'n / r*' mechanism)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>- Book derivation: Ch7 §7.1 equation (3) p.213; Figures 7.1 and 7.2; Appendix N net-transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>- Related external: Mage (1963) productive-capitalist-sector accounting (Appendix M validates the NIPA-based approach against Mage); Bowles &amp; Gintis (1985 critique of social wage); ST 1987 social-wage paper (ES1101/ES1102/ES1103)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>## Provenance trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>- **Original research**: `Technical/research/AS001_research.json`, researcher `agent`, 2026-05-16; verbatim quotes added 2026-05-23 (`stage1_cohort3_S901AS001AS002`) — sourced from chunk_24 (Ch7 §7.1 definitional and Figure 7.1) and chunk_38 (Appendix N net-transfer concept)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>- **DPR enriched**: 2026-05-23 by Stage-3 cohort-1 ingestion agent (cohort agent 4); sources read = research JSON + KB chunks 24/35/38 + registry entry + project CLAUDE.md (AS-prefix framing mandate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>- **Anu Framework stage**: Stage 3 INGESTION (cohort 1, failing chapters); ingestion gate IDs P31/P32</t>
         </is>
       </c>
     </row>
@@ -1212,13 +1405,299 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No research JSON for AS001</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>entry_id_or_type</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>content_or_quote</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>source_ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>verbatim_quote</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Divide equation (1) by utilized capital K*.u: r'n = [1 - T/S* - Eu/S*][S*/(K*.u)] = (1-t-eu)r*' = (1-b)r*'. Where r*' = S*/(K*.u) = capacity utilization-adjusted Marxian rate of profit; r'n = Pn/(K*.u) = similarly adjusted NIPA-based net rate of profit; t = T/S* = tax share of surplus value; eu = Eu/S* = unproductive expenses share of surplus value; b = t + eu = social burden rate.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ST_1994</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>verbatim_quote</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Observed net rate of profit r'n will fall relative to Marxian general rate r*' when greater proportion of surplus value absorbed in business taxes or unproductive expenses. Hence: b = social burden rate.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ST_1994</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>verbatim_quote</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Figure 7.1 shows the corresponding rise of 16% in social burden rate b over postwar period. Figure 7.2 result: NIPA-based rate rn falls substantially faster than Marxian rate. Marxian rate falls 25%, NIPA-based rate falls 39%.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ST_1994</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>verbatim_quote</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Net transfer: NT = Benefits received by workers - Taxes paid by workers. Purpose: Measure net impact of state expenditures and taxes on standard of living of wage/salary earners. Finding: Net transfer is negative over most of 1952-85 period -&gt; net tax on workers.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ST_1994</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>methodology_derived</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AS001 is a derived analytical series computing the Social Burden Rate. It is constructed from Net Social Wage (NSW, S607) and exploitation-related series. The social burden rate measures the proportion of surplus value absorbed by the net fiscal impact on workers — i.e., taxes paid by workers minus benefits and services received.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>series_registry.json (AS001 definition)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>construction_reference</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Registry describes AS001 as 'derived from NSW + exploitation series' with source_type 'analytical'. The legacy construction script is A07_social_burden_rate.py. Units are ratio. The series covers 1948-2024.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>series_registry.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>construction_reference</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>The social burden rate conceptually relates to Chapter 6's analysis of the net social wage (S607 = B_w + G_w - T_w) and its ratio to variable capital or surplus value. AS001 likely computes NSW relative to an exploitation measure (e.g., S*/V* or similar), quantifying the net fiscal redistribution burden on the surplus.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ST_1994, Ch6 concepts; series_registry.json cross-references</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>construction_reference</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Key input series: S607 (Net Social Wage), plus exploitation/surplus value series from Chapter 5 (e.g., S506 rate of surplus value, S505 surplus value). The construction array in the registry is empty, indicating this was handled by a standalone analytical script rather than the standard pipeline.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>series_registry.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>VERBATIM QUOTES (top-level)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>352-353</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>methodology_summary</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Derived analytical ratio measuring the social burden rate, computed from Net Social Wage (S607) and exploitation-related series. Legacy script: A07_social_burden_rate.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>known_issues:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Construction steps not specified in registry (empty array) — relies on legacy script</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Exact formula not yet verified against book text</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cross_references:</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>S607</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>S506</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>S505</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>citations:</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ST_1994</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Shaikh, Anwar, and E. Ahmet Tonak. 1994. Measuring the Wealth of Nations: The Political Economy of National Accounts. Cambridge University Press.</t>
         </is>
       </c>
     </row>
@@ -1233,11 +1712,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -1279,7 +1758,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>null — series does not extend beyond book period</t>
+          <t>null - series does not extend beyond book period</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1779,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"1948": 0.7906295851674003, "1958": 0.8287839156744095, "1970": 0.8425256084868625, "1980": 0.8474560743829904, "1989": 0.8577410093940578}</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1791,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>[0.3, 0.95]</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1803,43 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rate_series</t>
+          <t>share_series</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tolerance_class</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>share_series</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tolerance_rel</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tolerance_abs</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.01</t>
         </is>
       </c>
     </row>

</xml_diff>